<commit_message>
31 march 2026 updated
</commit_message>
<xml_diff>
--- a/Nooriemaan_March_2026_Attendance.xlsx
+++ b/Nooriemaan_March_2026_Attendance.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="22527"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_1C34990903B0C4446FF88A0432A8FCE9F3DFE88B" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{F11C4648-504F-4314-B8B6-B171BBB12FF3}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_1C34990903B0C4446FF88A0432A8FCE9F3DFE88B" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{2FAF6C14-2FD9-4457-A42D-D6645736A644}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="56">
   <si>
     <t>🕌  NOORIEMAAN DIGITAL PORTAL</t>
   </si>
@@ -139,9 +139,6 @@
     <t>16-Mar-2026</t>
   </si>
   <si>
-    <t>17-Mar-2026</t>
-  </si>
-  <si>
     <t>18-Mar-2026</t>
   </si>
   <si>
@@ -151,21 +148,6 @@
     <t>20-Mar-2026</t>
   </si>
   <si>
-    <t>21-Mar-2026</t>
-  </si>
-  <si>
-    <t>22-Mar-2026</t>
-  </si>
-  <si>
-    <t>23-Mar-2026</t>
-  </si>
-  <si>
-    <t>Pakistan Day 🇵🇰</t>
-  </si>
-  <si>
-    <t>24-Mar-2026</t>
-  </si>
-  <si>
     <t>25-Mar-2026</t>
   </si>
   <si>
@@ -190,19 +172,25 @@
     <t>📊  Summary</t>
   </si>
   <si>
-    <t>Working Days:  25</t>
-  </si>
-  <si>
-    <t>Holidays:  6</t>
-  </si>
-  <si>
-    <t>Filled:  0 / 25</t>
-  </si>
-  <si>
     <t>Generated: 2 March 2026   |   Nooriemaan Digital Portal   |   © Hanzalah Tahir</t>
   </si>
   <si>
     <t>Work</t>
+  </si>
+  <si>
+    <t>EID-UL-FITR</t>
+  </si>
+  <si>
+    <t>Weekly Off,EID-UL-FITR</t>
+  </si>
+  <si>
+    <t>Holidays:  8</t>
+  </si>
+  <si>
+    <t>Filled:  23 / 23</t>
+  </si>
+  <si>
+    <t>Working Days:  23</t>
   </si>
 </sst>
 </file>
@@ -358,7 +346,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -368,6 +356,21 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -382,19 +385,10 @@
       <alignment horizontal="right" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="15" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="15" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -749,52 +743,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
     </row>
     <row r="2" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
     </row>
     <row r="3" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="7" t="s">
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
     </row>
     <row r="4" spans="1:8" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -859,15 +853,15 @@
         <v>18</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E7" s="13">
+        <v>50</v>
+      </c>
+      <c r="E7" s="4">
         <v>0.28888888888888892</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="4">
         <v>0.41666666666666669</v>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="4">
         <v>0.1277777777777778</v>
       </c>
       <c r="H7" s="3" t="s">
@@ -885,15 +879,15 @@
         <v>20</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="13">
+        <v>50</v>
+      </c>
+      <c r="E8" s="4">
         <v>0.20347222222222219</v>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="4">
         <v>0.3298611111111111</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="4">
         <v>0.12638888888888888</v>
       </c>
       <c r="H8" s="3" t="s">
@@ -911,15 +905,15 @@
         <v>22</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E9" s="13">
+        <v>50</v>
+      </c>
+      <c r="E9" s="4">
         <v>0.23194444444444443</v>
       </c>
-      <c r="F9" s="13">
+      <c r="F9" s="4">
         <v>0.3576388888888889</v>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="4">
         <v>0.12569444444444444</v>
       </c>
       <c r="H9" s="3" t="s">
@@ -937,15 +931,15 @@
         <v>24</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E10" s="13">
+        <v>50</v>
+      </c>
+      <c r="E10" s="4">
         <v>0.24097222222222223</v>
       </c>
-      <c r="F10" s="13">
+      <c r="F10" s="4">
         <v>0.36805555555555558</v>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="4">
         <v>0.12708333333333333</v>
       </c>
       <c r="H10" s="3" t="s">
@@ -963,15 +957,15 @@
         <v>26</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E11" s="13">
+        <v>50</v>
+      </c>
+      <c r="E11" s="4">
         <v>9.0972222222222218E-2</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="4">
         <v>0.21597222222222223</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="4">
         <v>0.12708333333333333</v>
       </c>
       <c r="H11" s="3" t="s">
@@ -989,16 +983,16 @@
         <v>28</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E12" s="4">
+        <v>0.43333333333333335</v>
+      </c>
+      <c r="F12" s="4">
+        <v>5.9027777777777783E-2</v>
+      </c>
+      <c r="G12" s="4">
+        <v>0.12569444444444444</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>15</v>
@@ -1041,16 +1035,16 @@
         <v>18</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0.23819444444444446</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0.36458333333333331</v>
+      </c>
+      <c r="G14" s="4">
+        <v>0.12638888888888888</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>15</v>
@@ -1067,16 +1061,16 @@
         <v>20</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E15" s="4">
+        <v>0.2902777777777778</v>
+      </c>
+      <c r="F15" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="G15" s="4">
+        <v>0.12638888888888888</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>15</v>
@@ -1093,16 +1087,16 @@
         <v>22</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E16" s="4">
+        <v>0.18888888888888888</v>
+      </c>
+      <c r="F16" s="4">
+        <v>0.31388888888888888</v>
+      </c>
+      <c r="G16" s="4">
+        <v>0.125</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>15</v>
@@ -1119,16 +1113,16 @@
         <v>24</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E17" s="4">
+        <v>0.14166666666666666</v>
+      </c>
+      <c r="F17" s="4">
+        <v>0.2673611111111111</v>
+      </c>
+      <c r="G17" s="4">
+        <v>0.12569444444444444</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>15</v>
@@ -1145,16 +1139,16 @@
         <v>26</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E18" s="4">
+        <v>0.10416666666666667</v>
+      </c>
+      <c r="F18" s="4">
+        <v>0.22916666666666666</v>
+      </c>
+      <c r="G18" s="4">
+        <v>0.125</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>15</v>
@@ -1171,16 +1165,16 @@
         <v>28</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0.13333333333333333</v>
+      </c>
+      <c r="F19" s="4">
+        <v>0.25833333333333336</v>
+      </c>
+      <c r="G19" s="4">
+        <v>0.125</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>15</v>
@@ -1223,16 +1217,16 @@
         <v>18</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E21" s="4">
+        <v>0.20277777777777781</v>
+      </c>
+      <c r="F21" s="4">
+        <v>0.36944444444444446</v>
+      </c>
+      <c r="G21" s="4">
+        <v>0.125</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>15</v>
@@ -1242,23 +1236,23 @@
       <c r="A22" s="3">
         <v>17</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>38</v>
+      <c r="B22" s="15">
+        <v>46098</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E22" s="4">
+        <v>0.11944444444444445</v>
+      </c>
+      <c r="F22" s="4">
+        <v>0.24444444444444446</v>
+      </c>
+      <c r="G22" s="4">
+        <v>0.125</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>15</v>
@@ -1269,22 +1263,22 @@
         <v>18</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E23" s="4">
+        <v>0.24930555555555556</v>
+      </c>
+      <c r="F23" s="4">
+        <v>0.375</v>
+      </c>
+      <c r="G23" s="4">
+        <v>0.12569444444444444</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>15</v>
@@ -1295,22 +1289,22 @@
         <v>19</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E24" s="4">
+        <v>0.16944444444444443</v>
+      </c>
+      <c r="F24" s="4">
+        <v>0.29444444444444445</v>
+      </c>
+      <c r="G24" s="4">
+        <v>0.125</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>15</v>
@@ -1321,59 +1315,59 @@
         <v>20</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>26</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E25" s="4">
+        <v>0.2986111111111111</v>
+      </c>
+      <c r="F25" s="4">
+        <v>0.4236111111111111</v>
+      </c>
+      <c r="G25" s="4">
+        <v>0.125</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="3">
+      <c r="A26" s="2">
         <v>21</v>
       </c>
-      <c r="B26" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" s="3" t="s">
+      <c r="B26" s="14">
+        <v>46102</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G26" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>15</v>
+      <c r="D26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>22</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>43</v>
+      <c r="B27" s="14">
+        <v>46103</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>13</v>
@@ -1391,15 +1385,15 @@
         <v>15</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>16</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>23</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>44</v>
+      <c r="B28" s="14">
+        <v>46104</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>18</v>
@@ -1417,33 +1411,33 @@
         <v>15</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="3">
+      <c r="A29" s="2">
         <v>24</v>
       </c>
-      <c r="B29" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C29" s="3" t="s">
+      <c r="B29" s="14">
+        <v>46105</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>15</v>
+      <c r="D29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1451,22 +1445,22 @@
         <v>25</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G30" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E30" s="4">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="F30" s="4">
+        <v>0.19166666666666665</v>
+      </c>
+      <c r="G30" s="4">
+        <v>0.125</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>15</v>
@@ -1477,22 +1471,22 @@
         <v>26</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E31" s="4">
+        <v>9.3055555555555558E-2</v>
+      </c>
+      <c r="F31" s="4">
+        <v>0.21875</v>
+      </c>
+      <c r="G31" s="4">
+        <v>0.12569444444444444</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>15</v>
@@ -1503,22 +1497,22 @@
         <v>27</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>26</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G32" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E32" s="4">
+        <v>0.1423611111111111</v>
+      </c>
+      <c r="F32" s="4">
+        <v>0.2673611111111111</v>
+      </c>
+      <c r="G32" s="4">
+        <v>0.125</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>15</v>
@@ -1529,22 +1523,22 @@
         <v>28</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>28</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>15</v>
+        <v>50</v>
+      </c>
+      <c r="E33" s="4">
+        <v>0.10069444444444443</v>
+      </c>
+      <c r="F33" s="4">
+        <v>0.22569444444444445</v>
+      </c>
+      <c r="G33" s="4">
+        <v>0.125</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>15</v>
@@ -1555,7 +1549,7 @@
         <v>29</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>13</v>
@@ -1563,9 +1557,7 @@
       <c r="D34" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="E34" s="2"/>
       <c r="F34" s="2" t="s">
         <v>15</v>
       </c>
@@ -1581,13 +1573,13 @@
         <v>30</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>15</v>
@@ -1607,13 +1599,13 @@
         <v>31</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>15</v>
@@ -1630,48 +1622,48 @@
     </row>
     <row r="37" spans="1:8" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="1:8" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
+      <c r="A38" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B38" s="5"/>
+      <c r="C38" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D38" s="6"/>
+      <c r="E38" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F38" s="7"/>
+      <c r="G38" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B38" s="9"/>
-      <c r="C38" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="D38" s="10"/>
-      <c r="E38" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="F38" s="11"/>
-      <c r="G38" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="H38" s="10"/>
+      <c r="H38" s="6"/>
     </row>
     <row r="39" spans="1:8" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="B40" s="12"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
-      <c r="H40" s="12"/>
+      <c r="A40" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="8"/>
+      <c r="H40" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="A4:H4"/>
     <mergeCell ref="A38:B38"/>
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="E38:F38"/>
     <mergeCell ref="G38:H38"/>
     <mergeCell ref="A40:H40"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="A4:H4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>

<commit_message>
1 april 2026 updated
</commit_message>
<xml_diff>
--- a/Nooriemaan_March_2026_Attendance.xlsx
+++ b/Nooriemaan_March_2026_Attendance.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="22527"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_1C34990903B0C4446FF88A0432A8FCE9F3DFE88B" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{2FAF6C14-2FD9-4457-A42D-D6645736A644}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_1C34990903B0C4446FF88A0432A8FCE9F3DFE88B" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{55C63523-D686-4D17-BFD8-F15451D6C6DD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="56">
   <si>
     <t>🕌  NOORIEMAAN DIGITAL PORTAL</t>
   </si>
@@ -360,17 +360,11 @@
     <xf numFmtId="20" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="15" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="15" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -385,11 +379,17 @@
       <alignment horizontal="right" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="15" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="15" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -730,6 +730,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -743,52 +746,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
     </row>
     <row r="2" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
     </row>
     <row r="3" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="12" t="s">
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
     </row>
     <row r="4" spans="1:8" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
     </row>
     <row r="5" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -1236,7 +1239,7 @@
       <c r="A22" s="3">
         <v>17</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="6">
         <v>46098</v>
       </c>
       <c r="C22" s="3" t="s">
@@ -1340,7 +1343,7 @@
       <c r="A26" s="2">
         <v>21</v>
       </c>
-      <c r="B26" s="14">
+      <c r="B26" s="5">
         <v>46102</v>
       </c>
       <c r="C26" s="2" t="s">
@@ -1366,7 +1369,7 @@
       <c r="A27" s="2">
         <v>22</v>
       </c>
-      <c r="B27" s="14">
+      <c r="B27" s="5">
         <v>46103</v>
       </c>
       <c r="C27" s="2" t="s">
@@ -1392,7 +1395,7 @@
       <c r="A28" s="2">
         <v>23</v>
       </c>
-      <c r="B28" s="14">
+      <c r="B28" s="5">
         <v>46104</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -1418,7 +1421,7 @@
       <c r="A29" s="2">
         <v>24</v>
       </c>
-      <c r="B29" s="14">
+      <c r="B29" s="5">
         <v>46105</v>
       </c>
       <c r="C29" s="2" t="s">
@@ -1581,14 +1584,14 @@
       <c r="D35" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E35" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G35" s="3" t="s">
-        <v>15</v>
+      <c r="E35" s="4">
+        <v>0.2298611111111111</v>
+      </c>
+      <c r="F35" s="4">
+        <v>0.3576388888888889</v>
+      </c>
+      <c r="G35" s="4">
+        <v>0.1277777777777778</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>15</v>
@@ -1607,14 +1610,14 @@
       <c r="D36" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E36" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>15</v>
+      <c r="E36" s="4">
+        <v>0.29097222222222224</v>
+      </c>
+      <c r="F36" s="4">
+        <v>0.4201388888888889</v>
+      </c>
+      <c r="G36" s="4">
+        <v>0.12916666666666668</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>15</v>
@@ -1622,50 +1625,50 @@
     </row>
     <row r="37" spans="1:8" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="1:8" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B38" s="5"/>
-      <c r="C38" s="6" t="s">
+      <c r="B38" s="12"/>
+      <c r="C38" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="D38" s="6"/>
-      <c r="E38" s="7" t="s">
+      <c r="D38" s="13"/>
+      <c r="E38" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F38" s="7"/>
-      <c r="G38" s="6" t="s">
+      <c r="F38" s="14"/>
+      <c r="G38" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="H38" s="6"/>
+      <c r="H38" s="13"/>
     </row>
     <row r="39" spans="1:8" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="8" t="s">
+      <c r="A40" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="B40" s="8"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="8"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+      <c r="H40" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="A40:H40"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="E3:H3"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="A40:H40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup scale="48" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>